<commit_message>
se agrega avances scrum
</commit_message>
<xml_diff>
--- a/01_proyecto/trim1/01_contextualizacion_proyecto/PL01 - Plantilla de Definición.xlsx
+++ b/01_proyecto/trim1/01_contextualizacion_proyecto/PL01 - Plantilla de Definición.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AZUS\Desktop\hola\Innovation_Fusion\01_proyecto\trim1\01_contextualizacion_proyecto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E44D7A5E-0DBD-40B3-92BF-25A5AE879B89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E1EEFEB-2C38-4485-9671-A4BD5EDAADB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="15000" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="15000" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Equipo" sheetId="1" r:id="rId1"/>
@@ -623,7 +623,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -675,6 +675,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFA4C2F4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -819,7 +825,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -859,9 +865,6 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -883,6 +886,9 @@
     <xf numFmtId="0" fontId="10" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -901,6 +907,8 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -2367,15 +2375,15 @@
       </c>
     </row>
     <row r="4" spans="2:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="17"/>
-      <c r="H4" s="17"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="24"/>
     </row>
     <row r="5" spans="2:8" ht="175.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="8" t="s">
@@ -2493,15 +2501,15 @@
       </c>
     </row>
     <row r="10" spans="2:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="24" t="s">
         <v>55</v>
       </c>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24"/>
     </row>
     <row r="11" spans="2:8" ht="175.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="8" t="s">
@@ -2665,15 +2673,15 @@
       </c>
     </row>
     <row r="18" spans="2:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="24" t="s">
         <v>84</v>
       </c>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="17"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="24"/>
+      <c r="H18" s="24"/>
     </row>
     <row r="19" spans="2:8" ht="175.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="9" t="s">
@@ -2745,15 +2753,15 @@
       </c>
     </row>
     <row r="22" spans="2:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="17" t="s">
+      <c r="B22" s="24" t="s">
         <v>95</v>
       </c>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="17"/>
-      <c r="F22" s="17"/>
-      <c r="G22" s="17"/>
-      <c r="H22" s="17"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="24"/>
+      <c r="H22" s="24"/>
     </row>
     <row r="23" spans="2:8" ht="175.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="9" t="s">
@@ -2779,15 +2787,15 @@
       </c>
     </row>
     <row r="24" spans="2:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="17" t="s">
+      <c r="B24" s="24" t="s">
         <v>99</v>
       </c>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="17"/>
-      <c r="G24" s="17"/>
-      <c r="H24" s="17"/>
+      <c r="C24" s="24"/>
+      <c r="D24" s="24"/>
+      <c r="E24" s="24"/>
+      <c r="F24" s="24"/>
+      <c r="G24" s="24"/>
+      <c r="H24" s="24"/>
     </row>
     <row r="25" spans="2:8" ht="175.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="9" t="s">
@@ -2997,15 +3005,15 @@
       </c>
     </row>
     <row r="34" spans="2:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B34" s="17" t="s">
+      <c r="B34" s="24" t="s">
         <v>128</v>
       </c>
-      <c r="C34" s="17"/>
-      <c r="D34" s="17"/>
-      <c r="E34" s="17"/>
-      <c r="F34" s="17"/>
-      <c r="G34" s="17"/>
-      <c r="H34" s="17"/>
+      <c r="C34" s="24"/>
+      <c r="D34" s="24"/>
+      <c r="E34" s="24"/>
+      <c r="F34" s="24"/>
+      <c r="G34" s="24"/>
+      <c r="H34" s="24"/>
     </row>
     <row r="35" spans="2:8" ht="175.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B35" s="9" t="s">
@@ -3100,15 +3108,15 @@
       </c>
     </row>
     <row r="39" spans="2:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B39" s="17" t="s">
+      <c r="B39" s="24" t="s">
         <v>141</v>
       </c>
-      <c r="C39" s="17"/>
-      <c r="D39" s="17"/>
-      <c r="E39" s="17"/>
-      <c r="F39" s="17"/>
-      <c r="G39" s="17"/>
-      <c r="H39" s="17"/>
+      <c r="C39" s="24"/>
+      <c r="D39" s="24"/>
+      <c r="E39" s="24"/>
+      <c r="F39" s="24"/>
+      <c r="G39" s="24"/>
+      <c r="H39" s="24"/>
     </row>
     <row r="40" spans="2:8" ht="175.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B40" s="9" t="s">
@@ -3157,15 +3165,15 @@
       </c>
     </row>
     <row r="42" spans="2:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B42" s="17" t="s">
+      <c r="B42" s="24" t="s">
         <v>148</v>
       </c>
-      <c r="C42" s="17"/>
-      <c r="D42" s="17"/>
-      <c r="E42" s="17"/>
-      <c r="F42" s="17"/>
-      <c r="G42" s="17"/>
-      <c r="H42" s="17"/>
+      <c r="C42" s="24"/>
+      <c r="D42" s="24"/>
+      <c r="E42" s="24"/>
+      <c r="F42" s="24"/>
+      <c r="G42" s="24"/>
+      <c r="H42" s="24"/>
     </row>
     <row r="43" spans="2:8" ht="175.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B43" s="9" t="s">
@@ -3191,15 +3199,15 @@
       </c>
     </row>
     <row r="44" spans="2:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B44" s="17" t="s">
+      <c r="B44" s="24" t="s">
         <v>152</v>
       </c>
-      <c r="C44" s="17"/>
-      <c r="D44" s="17"/>
-      <c r="E44" s="17"/>
-      <c r="F44" s="17"/>
-      <c r="G44" s="17"/>
-      <c r="H44" s="17"/>
+      <c r="C44" s="24"/>
+      <c r="D44" s="24"/>
+      <c r="E44" s="24"/>
+      <c r="F44" s="24"/>
+      <c r="G44" s="24"/>
+      <c r="H44" s="24"/>
     </row>
     <row r="45" spans="2:8" ht="175.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B45" s="9" t="s">
@@ -4205,57 +4213,126 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82D6B611-C79A-4628-842F-788DD2B12556}">
-  <dimension ref="A1:AG38"/>
+  <dimension ref="A1:AJ38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="9.28515625" customWidth="1"/>
+    <col min="2" max="2" width="10.85546875" customWidth="1"/>
     <col min="3" max="3" width="7.42578125" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:36" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
-      <c r="L1" s="11"/>
-      <c r="M1" s="11"/>
-      <c r="N1" s="11"/>
-      <c r="O1" s="11"/>
-      <c r="P1" s="11"/>
-      <c r="Q1" s="11"/>
-      <c r="R1" s="11"/>
-      <c r="S1" s="11"/>
-      <c r="T1" s="11"/>
-      <c r="U1" s="11"/>
-      <c r="V1" s="11"/>
-      <c r="W1" s="11"/>
-      <c r="X1" s="11"/>
-      <c r="Y1" s="11"/>
-      <c r="Z1" s="11"/>
-      <c r="AA1" s="11"/>
-      <c r="AB1" s="11"/>
-      <c r="AC1" s="11"/>
-      <c r="AD1" s="11"/>
-      <c r="AE1" s="11"/>
-      <c r="AF1" s="11"/>
-      <c r="AG1" s="11"/>
-    </row>
-    <row r="2" spans="1:33" ht="42.75" x14ac:dyDescent="0.2">
+      <c r="D1" s="31">
+        <v>45979</v>
+      </c>
+      <c r="E1" s="31">
+        <v>45980</v>
+      </c>
+      <c r="F1" s="31">
+        <v>45981</v>
+      </c>
+      <c r="G1" s="31">
+        <v>45982</v>
+      </c>
+      <c r="H1" s="31">
+        <v>45983</v>
+      </c>
+      <c r="I1" s="31">
+        <v>45984</v>
+      </c>
+      <c r="J1" s="31">
+        <v>45985</v>
+      </c>
+      <c r="K1" s="31">
+        <v>45986</v>
+      </c>
+      <c r="L1" s="31">
+        <v>45987</v>
+      </c>
+      <c r="M1" s="31">
+        <v>45988</v>
+      </c>
+      <c r="N1" s="31">
+        <v>45989</v>
+      </c>
+      <c r="O1" s="31">
+        <v>45990</v>
+      </c>
+      <c r="P1" s="31">
+        <v>45991</v>
+      </c>
+      <c r="Q1" s="31">
+        <v>45992</v>
+      </c>
+      <c r="R1" s="31">
+        <v>45993</v>
+      </c>
+      <c r="S1" s="31">
+        <v>45994</v>
+      </c>
+      <c r="T1" s="31">
+        <v>45995</v>
+      </c>
+      <c r="U1" s="31">
+        <v>45996</v>
+      </c>
+      <c r="V1" s="31">
+        <v>45997</v>
+      </c>
+      <c r="W1" s="31">
+        <v>45998</v>
+      </c>
+      <c r="X1" s="31">
+        <v>45999</v>
+      </c>
+      <c r="Y1" s="31">
+        <v>46000</v>
+      </c>
+      <c r="Z1" s="31">
+        <v>46001</v>
+      </c>
+      <c r="AA1" s="31">
+        <v>46002</v>
+      </c>
+      <c r="AB1" s="31">
+        <v>46003</v>
+      </c>
+      <c r="AC1" s="31">
+        <v>46004</v>
+      </c>
+      <c r="AD1" s="31">
+        <v>46005</v>
+      </c>
+      <c r="AE1" s="31">
+        <v>46006</v>
+      </c>
+      <c r="AF1" s="31">
+        <v>46007</v>
+      </c>
+      <c r="AG1" s="31">
+        <v>46008</v>
+      </c>
+      <c r="AH1" s="31">
+        <v>46009</v>
+      </c>
+      <c r="AI1" s="31">
+        <v>46010</v>
+      </c>
+      <c r="AJ1" s="31">
+        <v>46011</v>
+      </c>
+    </row>
+    <row r="2" spans="1:36" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
         <v>43</v>
       </c>
@@ -4292,7 +4369,7 @@
       <c r="AF2" s="11"/>
       <c r="AG2" s="11"/>
     </row>
-    <row r="3" spans="1:33" ht="28.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:36" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A3" s="9" t="s">
         <v>44</v>
       </c>
@@ -4329,7 +4406,7 @@
       <c r="AF3" s="11"/>
       <c r="AG3" s="11"/>
     </row>
-    <row r="4" spans="1:33" ht="28.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:36" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A4" s="8" t="s">
         <v>46</v>
       </c>
@@ -4366,7 +4443,7 @@
       <c r="AF4" s="11"/>
       <c r="AG4" s="11"/>
     </row>
-    <row r="5" spans="1:33" ht="42.75" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:36" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="s">
         <v>47</v>
       </c>
@@ -4403,7 +4480,7 @@
       <c r="AF5" s="11"/>
       <c r="AG5" s="11"/>
     </row>
-    <row r="6" spans="1:33" ht="28.5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:36" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A6" s="8" t="s">
         <v>48</v>
       </c>
@@ -4440,7 +4517,7 @@
       <c r="AF6" s="11"/>
       <c r="AG6" s="11"/>
     </row>
-    <row r="7" spans="1:33" ht="42.75" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:36" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A7" s="9" t="s">
         <v>56</v>
       </c>
@@ -4477,7 +4554,7 @@
       <c r="AF7" s="11"/>
       <c r="AG7" s="11"/>
     </row>
-    <row r="8" spans="1:33" ht="57" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:36" ht="57" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
         <v>63</v>
       </c>
@@ -4514,7 +4591,7 @@
       <c r="AF8" s="11"/>
       <c r="AG8" s="11"/>
     </row>
-    <row r="9" spans="1:33" ht="28.5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:36" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
         <v>67</v>
       </c>
@@ -4551,7 +4628,7 @@
       <c r="AF9" s="11"/>
       <c r="AG9" s="11"/>
     </row>
-    <row r="10" spans="1:33" ht="28.5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:36" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A10" s="8" t="s">
         <v>69</v>
       </c>
@@ -4588,7 +4665,7 @@
       <c r="AF10" s="11"/>
       <c r="AG10" s="11"/>
     </row>
-    <row r="11" spans="1:33" ht="42.75" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:36" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A11" s="8" t="s">
         <v>73</v>
       </c>
@@ -4625,7 +4702,7 @@
       <c r="AF11" s="11"/>
       <c r="AG11" s="11"/>
     </row>
-    <row r="12" spans="1:33" ht="57" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:36" ht="57" x14ac:dyDescent="0.2">
       <c r="A12" s="8" t="s">
         <v>76</v>
       </c>
@@ -4662,7 +4739,7 @@
       <c r="AF12" s="11"/>
       <c r="AG12" s="11"/>
     </row>
-    <row r="13" spans="1:33" ht="42.75" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:36" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A13" s="8" t="s">
         <v>80</v>
       </c>
@@ -4699,11 +4776,13 @@
       <c r="AF13" s="11"/>
       <c r="AG13" s="11"/>
     </row>
-    <row r="14" spans="1:33" ht="28.5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:36" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A14" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="B14" s="11"/>
+      <c r="B14" s="31">
+        <v>39583</v>
+      </c>
       <c r="C14" s="11"/>
       <c r="D14" s="11"/>
       <c r="E14" s="11"/>
@@ -4736,7 +4815,7 @@
       <c r="AF14" s="11"/>
       <c r="AG14" s="11"/>
     </row>
-    <row r="15" spans="1:33" ht="71.25" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:36" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A15" s="9" t="s">
         <v>90</v>
       </c>
@@ -4773,7 +4852,7 @@
       <c r="AF15" s="11"/>
       <c r="AG15" s="11"/>
     </row>
-    <row r="16" spans="1:33" ht="85.5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:36" ht="85.5" x14ac:dyDescent="0.2">
       <c r="A16" s="9" t="s">
         <v>93</v>
       </c>
@@ -6587,148 +6666,148 @@
   <sheetData>
     <row r="2" spans="2:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="2:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="18"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="18"/>
+      <c r="B3" s="17"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="17"/>
     </row>
     <row r="4" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="20"/>
-      <c r="C4" s="21" t="s">
+      <c r="B4" s="19"/>
+      <c r="C4" s="20" t="s">
         <v>157</v>
       </c>
-      <c r="D4" s="21" t="s">
+      <c r="D4" s="20" t="s">
         <v>158</v>
       </c>
-      <c r="E4" s="21" t="s">
+      <c r="E4" s="20" t="s">
         <v>159</v>
       </c>
-      <c r="F4" s="18"/>
+      <c r="F4" s="17"/>
     </row>
     <row r="5" spans="2:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="20"/>
-      <c r="C5" s="22"/>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
-      <c r="F5" s="18"/>
+      <c r="B5" s="19"/>
+      <c r="C5" s="21"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="17"/>
     </row>
     <row r="6" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="20"/>
+      <c r="B6" s="19"/>
       <c r="C6" s="25" t="s">
         <v>16</v>
       </c>
       <c r="D6" s="26"/>
       <c r="E6" s="27"/>
-      <c r="F6" s="18"/>
+      <c r="F6" s="17"/>
     </row>
     <row r="7" spans="2:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="20"/>
+      <c r="B7" s="19"/>
       <c r="C7" s="28"/>
       <c r="D7" s="29"/>
       <c r="E7" s="30"/>
-      <c r="F7" s="18"/>
-    </row>
-    <row r="8" spans="2:6" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="20"/>
-      <c r="C8" s="21" t="s">
+      <c r="F7" s="17"/>
+    </row>
+    <row r="8" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="19"/>
+      <c r="C8" s="20" t="s">
         <v>160</v>
       </c>
-      <c r="D8" s="21" t="s">
+      <c r="D8" s="20" t="s">
         <v>161</v>
       </c>
-      <c r="E8" s="21" t="s">
+      <c r="E8" s="20" t="s">
         <v>162</v>
       </c>
-      <c r="F8" s="18"/>
+      <c r="F8" s="17"/>
     </row>
     <row r="9" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="20"/>
-      <c r="C9" s="23">
+      <c r="B9" s="19"/>
+      <c r="C9" s="22">
         <v>5</v>
       </c>
-      <c r="D9" s="23">
+      <c r="D9" s="22">
         <v>5</v>
       </c>
-      <c r="E9" s="22"/>
-      <c r="F9" s="18"/>
+      <c r="E9" s="21"/>
+      <c r="F9" s="17"/>
     </row>
     <row r="10" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="20"/>
+      <c r="B10" s="19"/>
       <c r="C10" s="25" t="s">
         <v>163</v>
       </c>
       <c r="D10" s="26"/>
       <c r="E10" s="27"/>
-      <c r="F10" s="18"/>
+      <c r="F10" s="17"/>
     </row>
     <row r="11" spans="2:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="20"/>
-      <c r="C11" s="24" t="s">
+      <c r="B11" s="19"/>
+      <c r="C11" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="D11" s="24" t="s">
+      <c r="D11" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="E11" s="24" t="s">
+      <c r="E11" s="23" t="s">
         <v>164</v>
       </c>
-      <c r="F11" s="18"/>
+      <c r="F11" s="17"/>
     </row>
     <row r="12" spans="2:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="20"/>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="18"/>
+      <c r="B12" s="19"/>
+      <c r="C12" s="21"/>
+      <c r="D12" s="21"/>
+      <c r="E12" s="21"/>
+      <c r="F12" s="17"/>
     </row>
     <row r="13" spans="2:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="20"/>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="18"/>
+      <c r="B13" s="19"/>
+      <c r="C13" s="21"/>
+      <c r="D13" s="21"/>
+      <c r="E13" s="21"/>
+      <c r="F13" s="17"/>
     </row>
     <row r="14" spans="2:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="20"/>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="18"/>
+      <c r="B14" s="19"/>
+      <c r="C14" s="21"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="21"/>
+      <c r="F14" s="17"/>
     </row>
     <row r="15" spans="2:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="20"/>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="18"/>
-    </row>
-    <row r="16" spans="2:6" ht="30.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="20"/>
-      <c r="C16" s="21" t="s">
+      <c r="B15" s="19"/>
+      <c r="C15" s="21"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="21"/>
+      <c r="F15" s="17"/>
+    </row>
+    <row r="16" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="19"/>
+      <c r="C16" s="20" t="s">
         <v>165</v>
       </c>
-      <c r="D16" s="21" t="s">
+      <c r="D16" s="20" t="s">
         <v>166</v>
       </c>
-      <c r="E16" s="21" t="s">
+      <c r="E16" s="20" t="s">
         <v>159</v>
       </c>
-      <c r="F16" s="18"/>
+      <c r="F16" s="17"/>
     </row>
     <row r="17" spans="2:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="20"/>
-      <c r="C17" s="22"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22"/>
-      <c r="F17" s="18"/>
+      <c r="B17" s="19"/>
+      <c r="C17" s="21"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="21"/>
+      <c r="F17" s="17"/>
     </row>
     <row r="18" spans="2:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="18"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="18"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
se sube adelantos scrum
</commit_message>
<xml_diff>
--- a/01_proyecto/trim1/01_contextualizacion_proyecto/PL01 - Plantilla de Definición.xlsx
+++ b/01_proyecto/trim1/01_contextualizacion_proyecto/PL01 - Plantilla de Definición.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AZUS\Desktop\Innovation_Fusion\01_proyecto\trim1\01_contextualizacion_proyecto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{350B04CA-0AD3-43B7-BCBA-29F0D2C06655}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F829CC4C-4ECF-4E91-A7C0-9966A45CE2B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="8" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Equipo" sheetId="1" r:id="rId1"/>
@@ -18,19 +18,24 @@
     <sheet name="Historia de Usuario" sheetId="3" r:id="rId3"/>
     <sheet name="Gestión de Usuarios y Autentica" sheetId="6" r:id="rId4"/>
     <sheet name="Catálogo y Experiencia de Naveg" sheetId="7" r:id="rId5"/>
-    <sheet name="Gestión de Productos e Inventar" sheetId="5" r:id="rId6"/>
+    <sheet name="Gestión de Productos e Inventar" sheetId="8" r:id="rId6"/>
+    <sheet name="Gestión de Promociones" sheetId="9" r:id="rId7"/>
+    <sheet name="Carrito y Checkout" sheetId="10" r:id="rId8"/>
+    <sheet name="Gestión de Devoluciones" sheetId="11" r:id="rId9"/>
+    <sheet name="Atención y Soporte al Cliente" sheetId="12" r:id="rId10"/>
+    <sheet name="Reportes y Administración Avanz" sheetId="13" r:id="rId11"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId8" roundtripDataChecksum="+CJhT1B5jpkQwxSTxyNLk1YCzpn9UEauZYMdiwIpMNk="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId12" roundtripDataChecksum="+CJhT1B5jpkQwxSTxyNLk1YCzpn9UEauZYMdiwIpMNk="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1092" uniqueCount="187">
   <si>
     <t>#</t>
   </si>
@@ -589,6 +594,12 @@
   </si>
   <si>
     <t>HU_003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Configurar precios y descuentos de los productos </t>
+  </si>
+  <si>
+    <t>Atención y Soporte al Cliente</t>
   </si>
 </sst>
 </file>
@@ -925,6 +936,9 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -959,9 +973,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2388,6 +2399,322 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9F8147E-37D2-41AD-9965-F04F594ADC86}">
+  <dimension ref="B1:D16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="17.7109375" customWidth="1"/>
+    <col min="3" max="3" width="30.7109375" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="2:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="B2" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B3" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>186</v>
+      </c>
+      <c r="D3" s="12"/>
+    </row>
+    <row r="4" spans="2:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="B4" s="27" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="27"/>
+      <c r="D4" s="27"/>
+    </row>
+    <row r="5" spans="2:4" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B5" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+    </row>
+    <row r="6" spans="2:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="B6" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="B7" s="13">
+        <v>5</v>
+      </c>
+      <c r="C7" s="13">
+        <v>8</v>
+      </c>
+      <c r="D7" s="12"/>
+    </row>
+    <row r="8" spans="2:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="B8" s="27" t="s">
+        <v>155</v>
+      </c>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B9" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" ht="51" x14ac:dyDescent="0.2">
+      <c r="B10" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="B11" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="B12" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="B13" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="14" spans="2:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="B14" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B15" s="12"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12"/>
+    </row>
+    <row r="16" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B16" s="16"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="16"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B8:D8"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{218130F5-64A5-4982-AF5F-1C1575E940E3}">
+  <dimension ref="B1:D16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="17.7109375" customWidth="1"/>
+    <col min="3" max="3" width="30.7109375" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="2:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="B2" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B3" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="D3" s="12"/>
+    </row>
+    <row r="4" spans="2:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="B4" s="27" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="27"/>
+      <c r="D4" s="27"/>
+    </row>
+    <row r="5" spans="2:4" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B5" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+    </row>
+    <row r="6" spans="2:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="B6" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="B7" s="13">
+        <v>5</v>
+      </c>
+      <c r="C7" s="13">
+        <v>8</v>
+      </c>
+      <c r="D7" s="12"/>
+    </row>
+    <row r="8" spans="2:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="B8" s="27" t="s">
+        <v>155</v>
+      </c>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B9" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" ht="51" x14ac:dyDescent="0.2">
+      <c r="B10" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="B11" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="B12" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="B13" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="14" spans="2:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="B14" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B15" s="12"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12"/>
+    </row>
+    <row r="16" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B16" s="16"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="16"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B8:D8"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
@@ -2430,15 +2757,15 @@
       </c>
     </row>
     <row r="4" spans="2:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
-      <c r="G4" s="16"/>
-      <c r="H4" s="16"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="17"/>
+      <c r="G4" s="17"/>
+      <c r="H4" s="17"/>
     </row>
     <row r="5" spans="2:8" ht="175.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="6" t="s">
@@ -2556,15 +2883,15 @@
       </c>
     </row>
     <row r="10" spans="2:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="16" t="s">
+      <c r="B10" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="C10" s="16"/>
-      <c r="D10" s="16"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="16"/>
-      <c r="G10" s="16"/>
-      <c r="H10" s="16"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="17"/>
     </row>
     <row r="11" spans="2:8" ht="175.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="6" t="s">
@@ -2728,15 +3055,15 @@
       </c>
     </row>
     <row r="18" spans="2:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="16" t="s">
+      <c r="B18" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="16"/>
-      <c r="H18" s="16"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="17"/>
     </row>
     <row r="19" spans="2:8" ht="175.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="7" t="s">
@@ -2808,15 +3135,15 @@
       </c>
     </row>
     <row r="22" spans="2:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="16" t="s">
+      <c r="B22" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="C22" s="16"/>
-      <c r="D22" s="16"/>
-      <c r="E22" s="16"/>
-      <c r="F22" s="16"/>
-      <c r="G22" s="16"/>
-      <c r="H22" s="16"/>
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="17"/>
+      <c r="F22" s="17"/>
+      <c r="G22" s="17"/>
+      <c r="H22" s="17"/>
     </row>
     <row r="23" spans="2:8" ht="175.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="7" t="s">
@@ -2842,15 +3169,15 @@
       </c>
     </row>
     <row r="24" spans="2:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="16" t="s">
+      <c r="B24" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="C24" s="16"/>
-      <c r="D24" s="16"/>
-      <c r="E24" s="16"/>
-      <c r="F24" s="16"/>
-      <c r="G24" s="16"/>
-      <c r="H24" s="16"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="17"/>
+      <c r="H24" s="17"/>
     </row>
     <row r="25" spans="2:8" ht="175.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="7" t="s">
@@ -3060,15 +3387,15 @@
       </c>
     </row>
     <row r="34" spans="2:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B34" s="16" t="s">
+      <c r="B34" s="17" t="s">
         <v>121</v>
       </c>
-      <c r="C34" s="16"/>
-      <c r="D34" s="16"/>
-      <c r="E34" s="16"/>
-      <c r="F34" s="16"/>
-      <c r="G34" s="16"/>
-      <c r="H34" s="16"/>
+      <c r="C34" s="17"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="17"/>
+      <c r="F34" s="17"/>
+      <c r="G34" s="17"/>
+      <c r="H34" s="17"/>
     </row>
     <row r="35" spans="2:8" ht="175.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B35" s="7" t="s">
@@ -3163,15 +3490,15 @@
       </c>
     </row>
     <row r="39" spans="2:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B39" s="16" t="s">
+      <c r="B39" s="17" t="s">
         <v>134</v>
       </c>
-      <c r="C39" s="16"/>
-      <c r="D39" s="16"/>
-      <c r="E39" s="16"/>
-      <c r="F39" s="16"/>
-      <c r="G39" s="16"/>
-      <c r="H39" s="16"/>
+      <c r="C39" s="17"/>
+      <c r="D39" s="17"/>
+      <c r="E39" s="17"/>
+      <c r="F39" s="17"/>
+      <c r="G39" s="17"/>
+      <c r="H39" s="17"/>
     </row>
     <row r="40" spans="2:8" ht="175.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B40" s="7" t="s">
@@ -3220,15 +3547,15 @@
       </c>
     </row>
     <row r="42" spans="2:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B42" s="16" t="s">
+      <c r="B42" s="17" t="s">
         <v>141</v>
       </c>
-      <c r="C42" s="16"/>
-      <c r="D42" s="16"/>
-      <c r="E42" s="16"/>
-      <c r="F42" s="16"/>
-      <c r="G42" s="16"/>
-      <c r="H42" s="16"/>
+      <c r="C42" s="17"/>
+      <c r="D42" s="17"/>
+      <c r="E42" s="17"/>
+      <c r="F42" s="17"/>
+      <c r="G42" s="17"/>
+      <c r="H42" s="17"/>
     </row>
     <row r="43" spans="2:8" ht="175.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B43" s="7" t="s">
@@ -3254,15 +3581,15 @@
       </c>
     </row>
     <row r="44" spans="2:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B44" s="16" t="s">
+      <c r="B44" s="17" t="s">
         <v>145</v>
       </c>
-      <c r="C44" s="16"/>
-      <c r="D44" s="16"/>
-      <c r="E44" s="16"/>
-      <c r="F44" s="16"/>
-      <c r="G44" s="16"/>
-      <c r="H44" s="16"/>
+      <c r="C44" s="17"/>
+      <c r="D44" s="17"/>
+      <c r="E44" s="17"/>
+      <c r="F44" s="17"/>
+      <c r="G44" s="17"/>
+      <c r="H44" s="17"/>
     </row>
     <row r="45" spans="2:8" ht="175.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B45" s="7" t="s">
@@ -4302,13 +4629,13 @@
       </c>
     </row>
     <row r="4" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="23"/>
     </row>
     <row r="5" spans="2:6" ht="61.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="9" t="s">
@@ -4398,13 +4725,13 @@
       <c r="F15" s="2"/>
     </row>
     <row r="16" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="17" t="s">
+      <c r="B16" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="19"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="20"/>
     </row>
     <row r="17" spans="2:6" ht="61.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="2"/>
@@ -4456,13 +4783,13 @@
       <c r="F23" s="2"/>
     </row>
     <row r="24" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="20" t="s">
+      <c r="B24" s="21" t="s">
         <v>77</v>
       </c>
-      <c r="C24" s="21"/>
-      <c r="D24" s="21"/>
-      <c r="E24" s="21"/>
-      <c r="F24" s="22"/>
+      <c r="C24" s="22"/>
+      <c r="D24" s="22"/>
+      <c r="E24" s="22"/>
+      <c r="F24" s="23"/>
     </row>
     <row r="25" spans="2:6" ht="61.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="9" t="s">
@@ -4512,13 +4839,13 @@
       <c r="F27" s="2"/>
     </row>
     <row r="28" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B28" s="23" t="s">
+      <c r="B28" s="24" t="s">
         <v>88</v>
       </c>
-      <c r="C28" s="24"/>
-      <c r="D28" s="24"/>
-      <c r="E28" s="24"/>
-      <c r="F28" s="25"/>
+      <c r="C28" s="25"/>
+      <c r="D28" s="25"/>
+      <c r="E28" s="25"/>
+      <c r="F28" s="26"/>
     </row>
     <row r="29" spans="2:6" ht="61.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="2"/>
@@ -4598,13 +4925,13 @@
       <c r="F39" s="2"/>
     </row>
     <row r="40" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B40" s="17" t="s">
+      <c r="B40" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="C40" s="18"/>
-      <c r="D40" s="18"/>
-      <c r="E40" s="18"/>
-      <c r="F40" s="19"/>
+      <c r="C40" s="19"/>
+      <c r="D40" s="19"/>
+      <c r="E40" s="19"/>
+      <c r="F40" s="20"/>
     </row>
     <row r="41" spans="2:6" ht="61.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B41" s="2"/>
@@ -4698,13 +5025,13 @@
       <c r="F53" s="2"/>
     </row>
     <row r="54" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B54" s="17" t="s">
+      <c r="B54" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="C54" s="18"/>
-      <c r="D54" s="18"/>
-      <c r="E54" s="18"/>
-      <c r="F54" s="19"/>
+      <c r="C54" s="19"/>
+      <c r="D54" s="19"/>
+      <c r="E54" s="19"/>
+      <c r="F54" s="20"/>
     </row>
     <row r="55" spans="2:6" ht="61.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B55" s="2"/>
@@ -4805,13 +5132,13 @@
       <c r="F68" s="2"/>
     </row>
     <row r="69" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B69" s="17" t="s">
+      <c r="B69" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="C69" s="18"/>
-      <c r="D69" s="18"/>
-      <c r="E69" s="18"/>
-      <c r="F69" s="19"/>
+      <c r="C69" s="19"/>
+      <c r="D69" s="19"/>
+      <c r="E69" s="19"/>
+      <c r="F69" s="20"/>
     </row>
     <row r="70" spans="2:6" ht="61.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B70" s="2"/>
@@ -4898,13 +5225,13 @@
       <c r="F81" s="2"/>
     </row>
     <row r="82" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B82" s="17" t="s">
+      <c r="B82" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="C82" s="18"/>
-      <c r="D82" s="18"/>
-      <c r="E82" s="18"/>
-      <c r="F82" s="19"/>
+      <c r="C82" s="19"/>
+      <c r="D82" s="19"/>
+      <c r="E82" s="19"/>
+      <c r="F82" s="20"/>
     </row>
     <row r="83" spans="2:6" ht="61.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B83" s="2"/>
@@ -4977,13 +5304,13 @@
       <c r="F92" s="2"/>
     </row>
     <row r="93" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B93" s="17" t="s">
+      <c r="B93" s="18" t="s">
         <v>145</v>
       </c>
-      <c r="C93" s="18"/>
-      <c r="D93" s="18"/>
-      <c r="E93" s="18"/>
-      <c r="F93" s="19"/>
+      <c r="C93" s="19"/>
+      <c r="D93" s="19"/>
+      <c r="E93" s="19"/>
+      <c r="F93" s="20"/>
     </row>
     <row r="94" spans="2:6" ht="61.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B94" s="2"/>
@@ -6048,60 +6375,60 @@
       <c r="T3" s="12"/>
     </row>
     <row r="4" spans="2:20" ht="15" x14ac:dyDescent="0.2">
-      <c r="B4" s="26" t="s">
+      <c r="B4" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="26"/>
-      <c r="D4" s="26"/>
-      <c r="F4" s="26" t="s">
+      <c r="C4" s="27"/>
+      <c r="D4" s="27"/>
+      <c r="F4" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="26"/>
-      <c r="H4" s="26"/>
-      <c r="J4" s="26" t="s">
+      <c r="G4" s="27"/>
+      <c r="H4" s="27"/>
+      <c r="J4" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="K4" s="26"/>
-      <c r="L4" s="26"/>
-      <c r="N4" s="26" t="s">
+      <c r="K4" s="27"/>
+      <c r="L4" s="27"/>
+      <c r="N4" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="O4" s="26"/>
-      <c r="P4" s="26"/>
-      <c r="R4" s="26" t="s">
+      <c r="O4" s="27"/>
+      <c r="P4" s="27"/>
+      <c r="R4" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="S4" s="26"/>
-      <c r="T4" s="26"/>
+      <c r="S4" s="27"/>
+      <c r="T4" s="27"/>
     </row>
     <row r="5" spans="2:20" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="27" t="s">
+      <c r="B5" s="28" t="s">
         <v>80</v>
       </c>
-      <c r="C5" s="27"/>
-      <c r="D5" s="27"/>
-      <c r="F5" s="27" t="s">
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="F5" s="28" t="s">
         <v>80</v>
       </c>
-      <c r="G5" s="27"/>
-      <c r="H5" s="27"/>
-      <c r="J5" s="27" t="s">
+      <c r="G5" s="28"/>
+      <c r="H5" s="28"/>
+      <c r="J5" s="28" t="s">
         <v>80</v>
       </c>
-      <c r="K5" s="27"/>
-      <c r="L5" s="27"/>
-      <c r="N5" s="27" t="s">
+      <c r="K5" s="28"/>
+      <c r="L5" s="28"/>
+      <c r="N5" s="28" t="s">
         <v>80</v>
       </c>
-      <c r="O5" s="27"/>
-      <c r="P5" s="27"/>
-      <c r="R5" s="27" t="s">
+      <c r="O5" s="28"/>
+      <c r="P5" s="28"/>
+      <c r="R5" s="28" t="s">
         <v>80</v>
       </c>
-      <c r="S5" s="27"/>
-      <c r="T5" s="27"/>
-    </row>
-    <row r="6" spans="2:20" ht="30" x14ac:dyDescent="0.2">
+      <c r="S5" s="28"/>
+      <c r="T5" s="28"/>
+    </row>
+    <row r="6" spans="2:20" ht="15" x14ac:dyDescent="0.2">
       <c r="B6" s="11" t="s">
         <v>152</v>
       </c>
@@ -6186,31 +6513,31 @@
       <c r="T7" s="12"/>
     </row>
     <row r="8" spans="2:20" ht="15" x14ac:dyDescent="0.2">
-      <c r="B8" s="26" t="s">
+      <c r="B8" s="27" t="s">
         <v>155</v>
       </c>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
-      <c r="F8" s="26" t="s">
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+      <c r="F8" s="27" t="s">
         <v>155</v>
       </c>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26"/>
-      <c r="J8" s="26" t="s">
+      <c r="G8" s="27"/>
+      <c r="H8" s="27"/>
+      <c r="J8" s="27" t="s">
         <v>155</v>
       </c>
-      <c r="K8" s="26"/>
-      <c r="L8" s="26"/>
-      <c r="N8" s="26" t="s">
+      <c r="K8" s="27"/>
+      <c r="L8" s="27"/>
+      <c r="N8" s="27" t="s">
         <v>155</v>
       </c>
-      <c r="O8" s="26"/>
-      <c r="P8" s="26"/>
-      <c r="R8" s="26" t="s">
+      <c r="O8" s="27"/>
+      <c r="P8" s="27"/>
+      <c r="R8" s="27" t="s">
         <v>155</v>
       </c>
-      <c r="S8" s="26"/>
-      <c r="T8" s="26"/>
+      <c r="S8" s="27"/>
+      <c r="T8" s="27"/>
     </row>
     <row r="9" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B9" s="14" t="s">
@@ -6259,7 +6586,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="10" spans="2:20" ht="76.5" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:20" ht="51" x14ac:dyDescent="0.2">
       <c r="B10" s="12" t="s">
         <v>169</v>
       </c>
@@ -6306,7 +6633,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="11" spans="2:20" ht="89.25" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:20" ht="63.75" x14ac:dyDescent="0.2">
       <c r="B11" s="12" t="s">
         <v>172</v>
       </c>
@@ -6353,7 +6680,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="12" spans="2:20" ht="127.5" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:20" ht="76.5" x14ac:dyDescent="0.2">
       <c r="B12" s="12" t="s">
         <v>173</v>
       </c>
@@ -6400,7 +6727,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="13" spans="2:20" ht="76.5" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:20" ht="38.25" x14ac:dyDescent="0.2">
       <c r="B13" s="12" t="s">
         <v>179</v>
       </c>
@@ -6447,7 +6774,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="14" spans="2:20" ht="30" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:20" ht="15" x14ac:dyDescent="0.2">
       <c r="B14" s="11" t="s">
         <v>157</v>
       </c>
@@ -6512,24 +6839,30 @@
       <c r="T15" s="12"/>
     </row>
     <row r="16" spans="2:20" x14ac:dyDescent="0.2">
-      <c r="B16" s="28"/>
-      <c r="C16" s="28"/>
-      <c r="D16" s="28"/>
-      <c r="F16" s="28"/>
-      <c r="G16" s="28"/>
-      <c r="H16" s="28"/>
-      <c r="J16" s="28"/>
-      <c r="K16" s="28"/>
-      <c r="L16" s="28"/>
-      <c r="N16" s="28"/>
-      <c r="O16" s="28"/>
-      <c r="P16" s="28"/>
-      <c r="R16" s="28"/>
-      <c r="S16" s="28"/>
-      <c r="T16" s="28"/>
+      <c r="B16" s="16"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="16"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="16"/>
+      <c r="J16" s="16"/>
+      <c r="K16" s="16"/>
+      <c r="L16" s="16"/>
+      <c r="N16" s="16"/>
+      <c r="O16" s="16"/>
+      <c r="P16" s="16"/>
+      <c r="R16" s="16"/>
+      <c r="S16" s="16"/>
+      <c r="T16" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="F5:H5"/>
+    <mergeCell ref="F8:H8"/>
     <mergeCell ref="R4:T4"/>
     <mergeCell ref="R5:T5"/>
     <mergeCell ref="R8:T8"/>
@@ -6539,12 +6872,6 @@
     <mergeCell ref="N4:P4"/>
     <mergeCell ref="N5:P5"/>
     <mergeCell ref="N8:P8"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="F4:H4"/>
-    <mergeCell ref="F5:H5"/>
-    <mergeCell ref="F8:H8"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6553,7 +6880,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30E03081-6D4B-48F0-9762-CB959C944999}">
-  <dimension ref="B2:T15"/>
+  <dimension ref="B2:T30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="17.7109375" customWidth="1"/>
@@ -6620,7 +6947,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="3" spans="2:20" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B3" s="12" t="s">
         <v>183</v>
       </c>
@@ -6658,60 +6985,60 @@
       <c r="T3" s="12"/>
     </row>
     <row r="4" spans="2:20" ht="15" x14ac:dyDescent="0.2">
-      <c r="B4" s="26" t="s">
+      <c r="B4" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="26"/>
-      <c r="D4" s="26"/>
-      <c r="F4" s="26" t="s">
+      <c r="C4" s="27"/>
+      <c r="D4" s="27"/>
+      <c r="F4" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="26"/>
-      <c r="H4" s="26"/>
-      <c r="J4" s="26" t="s">
+      <c r="G4" s="27"/>
+      <c r="H4" s="27"/>
+      <c r="J4" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="K4" s="26"/>
-      <c r="L4" s="26"/>
-      <c r="N4" s="26" t="s">
+      <c r="K4" s="27"/>
+      <c r="L4" s="27"/>
+      <c r="N4" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="O4" s="26"/>
-      <c r="P4" s="26"/>
-      <c r="R4" s="26" t="s">
+      <c r="O4" s="27"/>
+      <c r="P4" s="27"/>
+      <c r="R4" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="S4" s="26"/>
-      <c r="T4" s="26"/>
+      <c r="S4" s="27"/>
+      <c r="T4" s="27"/>
     </row>
     <row r="5" spans="2:20" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="27" t="s">
+      <c r="B5" s="28" t="s">
         <v>80</v>
       </c>
-      <c r="C5" s="27"/>
-      <c r="D5" s="27"/>
-      <c r="F5" s="27" t="s">
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="F5" s="28" t="s">
         <v>80</v>
       </c>
-      <c r="G5" s="27"/>
-      <c r="H5" s="27"/>
-      <c r="J5" s="27" t="s">
+      <c r="G5" s="28"/>
+      <c r="H5" s="28"/>
+      <c r="J5" s="28" t="s">
         <v>80</v>
       </c>
-      <c r="K5" s="27"/>
-      <c r="L5" s="27"/>
-      <c r="N5" s="27" t="s">
+      <c r="K5" s="28"/>
+      <c r="L5" s="28"/>
+      <c r="N5" s="28" t="s">
         <v>80</v>
       </c>
-      <c r="O5" s="27"/>
-      <c r="P5" s="27"/>
-      <c r="R5" s="27" t="s">
+      <c r="O5" s="28"/>
+      <c r="P5" s="28"/>
+      <c r="R5" s="28" t="s">
         <v>80</v>
       </c>
-      <c r="S5" s="27"/>
-      <c r="T5" s="27"/>
-    </row>
-    <row r="6" spans="2:20" ht="30" x14ac:dyDescent="0.2">
+      <c r="S5" s="28"/>
+      <c r="T5" s="28"/>
+    </row>
+    <row r="6" spans="2:20" ht="15" x14ac:dyDescent="0.2">
       <c r="B6" s="11" t="s">
         <v>152</v>
       </c>
@@ -6796,31 +7123,31 @@
       <c r="T7" s="12"/>
     </row>
     <row r="8" spans="2:20" ht="15" x14ac:dyDescent="0.2">
-      <c r="B8" s="26" t="s">
+      <c r="B8" s="27" t="s">
         <v>155</v>
       </c>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
-      <c r="F8" s="26" t="s">
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+      <c r="F8" s="27" t="s">
         <v>155</v>
       </c>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26"/>
-      <c r="J8" s="26" t="s">
+      <c r="G8" s="27"/>
+      <c r="H8" s="27"/>
+      <c r="J8" s="27" t="s">
         <v>155</v>
       </c>
-      <c r="K8" s="26"/>
-      <c r="L8" s="26"/>
-      <c r="N8" s="26" t="s">
+      <c r="K8" s="27"/>
+      <c r="L8" s="27"/>
+      <c r="N8" s="27" t="s">
         <v>155</v>
       </c>
-      <c r="O8" s="26"/>
-      <c r="P8" s="26"/>
-      <c r="R8" s="26" t="s">
+      <c r="O8" s="27"/>
+      <c r="P8" s="27"/>
+      <c r="R8" s="27" t="s">
         <v>155</v>
       </c>
-      <c r="S8" s="26"/>
-      <c r="T8" s="26"/>
+      <c r="S8" s="27"/>
+      <c r="T8" s="27"/>
     </row>
     <row r="9" spans="2:20" x14ac:dyDescent="0.2">
       <c r="B9" s="14" t="s">
@@ -6869,7 +7196,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="10" spans="2:20" ht="76.5" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:20" ht="51" x14ac:dyDescent="0.2">
       <c r="B10" s="12" t="s">
         <v>169</v>
       </c>
@@ -6916,7 +7243,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="11" spans="2:20" ht="89.25" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:20" ht="63.75" x14ac:dyDescent="0.2">
       <c r="B11" s="12" t="s">
         <v>172</v>
       </c>
@@ -6963,7 +7290,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="12" spans="2:20" ht="127.5" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:20" ht="76.5" x14ac:dyDescent="0.2">
       <c r="B12" s="12" t="s">
         <v>173</v>
       </c>
@@ -7010,7 +7337,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="13" spans="2:20" ht="76.5" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:20" ht="38.25" x14ac:dyDescent="0.2">
       <c r="B13" s="12" t="s">
         <v>179</v>
       </c>
@@ -7057,7 +7384,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="14" spans="2:20" ht="30" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:20" ht="15" x14ac:dyDescent="0.2">
       <c r="B14" s="11" t="s">
         <v>157</v>
       </c>
@@ -7121,178 +7448,2127 @@
       <c r="S15" s="12"/>
       <c r="T15" s="12"/>
     </row>
+    <row r="17" spans="2:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="B17" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="F17" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="G17" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="H17" s="11" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="B18" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="C18" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="D18" s="12"/>
+      <c r="F18" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="G18" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="H18" s="12"/>
+    </row>
+    <row r="19" spans="2:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="B19" s="27" t="s">
+        <v>16</v>
+      </c>
+      <c r="C19" s="27"/>
+      <c r="D19" s="27"/>
+      <c r="F19" s="27" t="s">
+        <v>16</v>
+      </c>
+      <c r="G19" s="27"/>
+      <c r="H19" s="27"/>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B20" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="C20" s="28"/>
+      <c r="D20" s="28"/>
+      <c r="F20" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="G20" s="28"/>
+      <c r="H20" s="28"/>
+    </row>
+    <row r="21" spans="2:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="B21" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="D21" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="F21" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="G21" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="H21" s="11" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="B22" s="13">
+        <v>5</v>
+      </c>
+      <c r="C22" s="13">
+        <v>8</v>
+      </c>
+      <c r="D22" s="12"/>
+      <c r="F22" s="13">
+        <v>5</v>
+      </c>
+      <c r="G22" s="13">
+        <v>8</v>
+      </c>
+      <c r="H22" s="12"/>
+    </row>
+    <row r="23" spans="2:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="B23" s="27" t="s">
+        <v>155</v>
+      </c>
+      <c r="C23" s="27"/>
+      <c r="D23" s="27"/>
+      <c r="F23" s="27" t="s">
+        <v>155</v>
+      </c>
+      <c r="G23" s="27"/>
+      <c r="H23" s="27"/>
+    </row>
+    <row r="24" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B24" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C24" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="D24" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="F24" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="G24" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="H24" s="14" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="25" spans="2:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="B25" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="D25" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="F25" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="G25" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="H25" s="12" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="26" spans="2:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="B26" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="D26" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="F26" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="G26" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="H26" s="12" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="27" spans="2:8" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="B27" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="D27" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="F27" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="G27" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="H27" s="12" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="28" spans="2:8" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="B28" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="C28" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>181</v>
+      </c>
+      <c r="F28" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="G28" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="H28" s="12" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="29" spans="2:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="B29" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="C29" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="D29" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="F29" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="G29" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="H29" s="11" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="30" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B30" s="12"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="12"/>
+      <c r="F30" s="12"/>
+      <c r="G30" s="12"/>
+      <c r="H30" s="12"/>
+    </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="21">
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="F20:H20"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="F23:H23"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="F8:H8"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="F19:H19"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="F5:H5"/>
+    <mergeCell ref="J5:L5"/>
+    <mergeCell ref="N5:P5"/>
+    <mergeCell ref="R5:T5"/>
     <mergeCell ref="J4:L4"/>
     <mergeCell ref="N4:P4"/>
     <mergeCell ref="R4:T4"/>
     <mergeCell ref="J8:L8"/>
     <mergeCell ref="N8:P8"/>
     <mergeCell ref="R8:T8"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="F5:H5"/>
-    <mergeCell ref="J5:L5"/>
-    <mergeCell ref="N5:P5"/>
-    <mergeCell ref="R5:T5"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="F8:H8"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="F4:H4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2D2BA1A-E3EC-4B05-B9AB-FCC72E25559E}">
-  <dimension ref="C4:E17"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{489E27E4-4C61-4BC4-AE36-B09E77141EC6}">
+  <dimension ref="B1:L16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="3.85546875" customWidth="1"/>
-    <col min="3" max="3" width="17.7109375" customWidth="1"/>
-    <col min="4" max="4" width="29.85546875" customWidth="1"/>
-    <col min="5" max="5" width="24.5703125" customWidth="1"/>
+    <col min="2" max="2" width="17.7109375" customWidth="1"/>
+    <col min="3" max="3" width="30.7109375" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" customWidth="1"/>
+    <col min="6" max="6" width="17.7109375" customWidth="1"/>
+    <col min="7" max="7" width="30.7109375" customWidth="1"/>
+    <col min="8" max="8" width="17.5703125" customWidth="1"/>
+    <col min="10" max="10" width="17.7109375" customWidth="1"/>
+    <col min="11" max="11" width="30.7109375" customWidth="1"/>
+    <col min="12" max="12" width="17.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="3:5" ht="15" x14ac:dyDescent="0.2">
-      <c r="C4" s="11" t="s">
+    <row r="1" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="2:12" ht="15" x14ac:dyDescent="0.2">
+      <c r="B2" s="11" t="s">
         <v>149</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="C2" s="11" t="s">
         <v>150</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="D2" s="11" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="5" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C5" s="12" t="s">
-        <v>162</v>
-      </c>
-      <c r="D5" s="15" t="s">
+      <c r="F2" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="H2" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="J2" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="K2" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="L2" s="11" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="3" spans="2:12" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="B3" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="C3" s="15" t="s">
         <v>79</v>
       </c>
-      <c r="E5" s="12"/>
-    </row>
-    <row r="6" spans="3:5" ht="15" x14ac:dyDescent="0.2">
-      <c r="C6" s="26" t="s">
+      <c r="D3" s="12"/>
+      <c r="F3" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="G3" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="H3" s="12"/>
+      <c r="J3" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="K3" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="L3" s="12"/>
+    </row>
+    <row r="4" spans="2:12" ht="15" x14ac:dyDescent="0.2">
+      <c r="B4" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="26"/>
-      <c r="E6" s="26"/>
-    </row>
-    <row r="7" spans="3:5" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C7" s="27" t="s">
+      <c r="C4" s="27"/>
+      <c r="D4" s="27"/>
+      <c r="F4" s="27" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="27"/>
+      <c r="H4" s="27"/>
+      <c r="J4" s="27" t="s">
+        <v>16</v>
+      </c>
+      <c r="K4" s="27"/>
+      <c r="L4" s="27"/>
+    </row>
+    <row r="5" spans="2:12" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B5" s="28" t="s">
         <v>80</v>
       </c>
-      <c r="D7" s="27"/>
-      <c r="E7" s="27"/>
-    </row>
-    <row r="8" spans="3:5" ht="15" x14ac:dyDescent="0.2">
-      <c r="C8" s="11" t="s">
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="F5" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="G5" s="28"/>
+      <c r="H5" s="28"/>
+      <c r="J5" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="K5" s="28"/>
+      <c r="L5" s="28"/>
+    </row>
+    <row r="6" spans="2:12" ht="15" x14ac:dyDescent="0.2">
+      <c r="B6" s="11" t="s">
         <v>152</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="C6" s="11" t="s">
         <v>153</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="D6" s="11" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="9" spans="3:5" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="C9" s="13">
+      <c r="F6" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="H6" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="J6" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="K6" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="L6" s="11" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="B7" s="13">
         <v>5</v>
       </c>
-      <c r="D9" s="13">
+      <c r="C7" s="13">
         <v>8</v>
       </c>
-      <c r="E9" s="12"/>
-    </row>
-    <row r="10" spans="3:5" ht="15" x14ac:dyDescent="0.2">
-      <c r="C10" s="26" t="s">
+      <c r="D7" s="12"/>
+      <c r="F7" s="13">
+        <v>5</v>
+      </c>
+      <c r="G7" s="13">
+        <v>8</v>
+      </c>
+      <c r="H7" s="12"/>
+      <c r="J7" s="13">
+        <v>5</v>
+      </c>
+      <c r="K7" s="13">
+        <v>8</v>
+      </c>
+      <c r="L7" s="12"/>
+    </row>
+    <row r="8" spans="2:12" ht="15" x14ac:dyDescent="0.2">
+      <c r="B8" s="27" t="s">
         <v>155</v>
       </c>
-      <c r="D10" s="26"/>
-      <c r="E10" s="26"/>
-    </row>
-    <row r="11" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C11" s="14" t="s">
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+      <c r="F8" s="27" t="s">
+        <v>155</v>
+      </c>
+      <c r="G8" s="27"/>
+      <c r="H8" s="27"/>
+      <c r="J8" s="27" t="s">
+        <v>155</v>
+      </c>
+      <c r="K8" s="27"/>
+      <c r="L8" s="27"/>
+    </row>
+    <row r="9" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B9" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="D11" s="14" t="s">
+      <c r="C9" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="E11" s="14" t="s">
+      <c r="D9" s="14" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="12" spans="3:5" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="F9" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="G9" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="H9" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="J9" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="K9" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="L9" s="14" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12" ht="51" x14ac:dyDescent="0.2">
+      <c r="B10" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="H10" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="J10" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="K10" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="L10" s="12" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12" ht="51" x14ac:dyDescent="0.2">
+      <c r="B11" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="G11" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="H11" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="J11" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="K11" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="L11" s="12" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="12" spans="2:12" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="B12" s="12" t="s">
+        <v>173</v>
+      </c>
       <c r="C12" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="G12" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="H12" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="J12" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="K12" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="L12" s="12" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="B13" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>181</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="G13" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="H13" s="12" t="s">
+        <v>181</v>
+      </c>
+      <c r="J13" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="K13" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="L13" s="12" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12" ht="15" x14ac:dyDescent="0.2">
+      <c r="B14" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="G14" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="H14" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="J14" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="K14" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="L14" s="11" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B15" s="12"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
+      <c r="J15" s="12"/>
+      <c r="K15" s="12"/>
+      <c r="L15" s="12"/>
+    </row>
+    <row r="16" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B16" s="16"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="16"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="16"/>
+      <c r="J16" s="16"/>
+      <c r="K16" s="16"/>
+      <c r="L16" s="16"/>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="F8:H8"/>
+    <mergeCell ref="J8:L8"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="F5:H5"/>
+    <mergeCell ref="J5:L5"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C3122D9-6023-4932-A010-29D00F97AB8B}">
+  <dimension ref="B1:D16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="17.7109375" customWidth="1"/>
+    <col min="3" max="3" width="30.7109375" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="2:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="B2" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="B3" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="D3" s="12"/>
+    </row>
+    <row r="4" spans="2:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="B4" s="27" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="27"/>
+      <c r="D4" s="27"/>
+    </row>
+    <row r="5" spans="2:4" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B5" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+    </row>
+    <row r="6" spans="2:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="B6" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="B7" s="13">
+        <v>5</v>
+      </c>
+      <c r="C7" s="13">
+        <v>8</v>
+      </c>
+      <c r="D7" s="12"/>
+    </row>
+    <row r="8" spans="2:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="B8" s="27" t="s">
+        <v>155</v>
+      </c>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B9" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" ht="51" x14ac:dyDescent="0.2">
+      <c r="B10" s="12" t="s">
         <v>169</v>
       </c>
+      <c r="C10" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" ht="51" x14ac:dyDescent="0.2">
+      <c r="B11" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="B12" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>171</v>
+      </c>
       <c r="D12" s="12" t="s">
-        <v>177</v>
-      </c>
-      <c r="E12" s="12" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="13" spans="3:5" ht="38.25" x14ac:dyDescent="0.2">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="B13" s="12" t="s">
+        <v>179</v>
+      </c>
       <c r="C13" s="12" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="E13" s="12" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="14" spans="3:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="C14" s="12" t="s">
-        <v>173</v>
-      </c>
-      <c r="D14" s="12" t="s">
-        <v>171</v>
-      </c>
-      <c r="E14" s="12" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="15" spans="3:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="C15" s="12" t="s">
-        <v>179</v>
-      </c>
-      <c r="D15" s="12" t="s">
-        <v>180</v>
-      </c>
-      <c r="E15" s="12" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="16" spans="3:5" ht="15" x14ac:dyDescent="0.2">
-      <c r="C16" s="11" t="s">
+    <row r="14" spans="2:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="B14" s="11" t="s">
         <v>157</v>
       </c>
-      <c r="D16" s="11" t="s">
+      <c r="C14" s="11" t="s">
         <v>158</v>
       </c>
-      <c r="E16" s="11" t="s">
+      <c r="D14" s="11" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="17" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
+    <row r="15" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B15" s="12"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12"/>
+    </row>
+    <row r="16" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B16" s="16"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="C6:E6"/>
-    <mergeCell ref="C7:E7"/>
-    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B5:D5"/>
   </mergeCells>
-  <phoneticPr fontId="12" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30FD71FA-6566-4507-8277-A0D58B677FEC}">
+  <dimension ref="B2:T30"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="17.7109375" customWidth="1"/>
+    <col min="3" max="3" width="30.7109375" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" customWidth="1"/>
+    <col min="5" max="5" width="11.5703125" customWidth="1"/>
+    <col min="6" max="6" width="17.7109375" customWidth="1"/>
+    <col min="7" max="7" width="30.7109375" customWidth="1"/>
+    <col min="8" max="8" width="17.5703125" customWidth="1"/>
+    <col min="10" max="11" width="30.7109375" customWidth="1"/>
+    <col min="12" max="12" width="17.5703125" customWidth="1"/>
+    <col min="14" max="14" width="17.7109375" customWidth="1"/>
+    <col min="15" max="15" width="30.7109375" customWidth="1"/>
+    <col min="16" max="16" width="17.5703125" customWidth="1"/>
+    <col min="18" max="18" width="17.7109375" customWidth="1"/>
+    <col min="19" max="19" width="30.7109375" customWidth="1"/>
+    <col min="20" max="20" width="17.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:20" ht="15" x14ac:dyDescent="0.2">
+      <c r="B2" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="H2" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="J2" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="K2" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="L2" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="N2" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="O2" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="P2" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="R2" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="S2" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="T2" s="11" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="3" spans="2:20" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="B3" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="D3" s="12"/>
+      <c r="F3" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="G3" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="H3" s="12"/>
+      <c r="J3" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="K3" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="L3" s="12"/>
+      <c r="N3" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="O3" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="P3" s="12"/>
+      <c r="R3" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="S3" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="T3" s="12"/>
+    </row>
+    <row r="4" spans="2:20" ht="15" x14ac:dyDescent="0.2">
+      <c r="B4" s="27" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="27"/>
+      <c r="D4" s="27"/>
+      <c r="F4" s="27" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="27"/>
+      <c r="H4" s="27"/>
+      <c r="J4" s="27" t="s">
+        <v>16</v>
+      </c>
+      <c r="K4" s="27"/>
+      <c r="L4" s="27"/>
+      <c r="N4" s="27" t="s">
+        <v>16</v>
+      </c>
+      <c r="O4" s="27"/>
+      <c r="P4" s="27"/>
+      <c r="R4" s="27" t="s">
+        <v>16</v>
+      </c>
+      <c r="S4" s="27"/>
+      <c r="T4" s="27"/>
+    </row>
+    <row r="5" spans="2:20" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B5" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="F5" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="G5" s="28"/>
+      <c r="H5" s="28"/>
+      <c r="J5" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="K5" s="28"/>
+      <c r="L5" s="28"/>
+      <c r="N5" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="O5" s="28"/>
+      <c r="P5" s="28"/>
+      <c r="R5" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="S5" s="28"/>
+      <c r="T5" s="28"/>
+    </row>
+    <row r="6" spans="2:20" ht="15" x14ac:dyDescent="0.2">
+      <c r="B6" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="H6" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="J6" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="K6" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="L6" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="N6" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="O6" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="P6" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="R6" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="S6" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="T6" s="11" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="7" spans="2:20" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="B7" s="13">
+        <v>5</v>
+      </c>
+      <c r="C7" s="13">
+        <v>8</v>
+      </c>
+      <c r="D7" s="12"/>
+      <c r="F7" s="13">
+        <v>5</v>
+      </c>
+      <c r="G7" s="13">
+        <v>8</v>
+      </c>
+      <c r="H7" s="12"/>
+      <c r="J7" s="13">
+        <v>5</v>
+      </c>
+      <c r="K7" s="13">
+        <v>8</v>
+      </c>
+      <c r="L7" s="12"/>
+      <c r="N7" s="13">
+        <v>5</v>
+      </c>
+      <c r="O7" s="13">
+        <v>8</v>
+      </c>
+      <c r="P7" s="12"/>
+      <c r="R7" s="13">
+        <v>5</v>
+      </c>
+      <c r="S7" s="13">
+        <v>8</v>
+      </c>
+      <c r="T7" s="12"/>
+    </row>
+    <row r="8" spans="2:20" ht="15" x14ac:dyDescent="0.2">
+      <c r="B8" s="27" t="s">
+        <v>155</v>
+      </c>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+      <c r="F8" s="27" t="s">
+        <v>155</v>
+      </c>
+      <c r="G8" s="27"/>
+      <c r="H8" s="27"/>
+      <c r="J8" s="27" t="s">
+        <v>155</v>
+      </c>
+      <c r="K8" s="27"/>
+      <c r="L8" s="27"/>
+      <c r="N8" s="27" t="s">
+        <v>155</v>
+      </c>
+      <c r="O8" s="27"/>
+      <c r="P8" s="27"/>
+      <c r="R8" s="27" t="s">
+        <v>155</v>
+      </c>
+      <c r="S8" s="27"/>
+      <c r="T8" s="27"/>
+    </row>
+    <row r="9" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B9" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="F9" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="G9" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="H9" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="J9" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="K9" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="L9" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="N9" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="O9" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="P9" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="R9" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="S9" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="T9" s="14" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="10" spans="2:20" ht="51" x14ac:dyDescent="0.2">
+      <c r="B10" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="H10" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="J10" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="K10" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="L10" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="N10" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="O10" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="P10" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="R10" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="S10" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="T10" s="12" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="11" spans="2:20" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="B11" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="G11" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="H11" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="J11" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="K11" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="L11" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="N11" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="O11" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="P11" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="R11" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="S11" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="T11" s="12" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="12" spans="2:20" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="B12" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="G12" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="H12" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="J12" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="K12" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="L12" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="N12" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="O12" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="P12" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="R12" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="S12" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="T12" s="12" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="13" spans="2:20" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="B13" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>181</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="G13" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="H13" s="12" t="s">
+        <v>181</v>
+      </c>
+      <c r="J13" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="K13" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="L13" s="12" t="s">
+        <v>181</v>
+      </c>
+      <c r="N13" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="O13" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="P13" s="12" t="s">
+        <v>181</v>
+      </c>
+      <c r="R13" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="S13" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="T13" s="12" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="14" spans="2:20" ht="15" x14ac:dyDescent="0.2">
+      <c r="B14" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="G14" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="H14" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="J14" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="K14" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="L14" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="N14" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="O14" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="P14" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="R14" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="S14" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="T14" s="11" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="15" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="B15" s="12"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
+      <c r="J15" s="12"/>
+      <c r="K15" s="12"/>
+      <c r="L15" s="12"/>
+      <c r="N15" s="12"/>
+      <c r="O15" s="12"/>
+      <c r="P15" s="12"/>
+      <c r="R15" s="12"/>
+      <c r="S15" s="12"/>
+      <c r="T15" s="12"/>
+    </row>
+    <row r="17" spans="2:16" ht="15" x14ac:dyDescent="0.2">
+      <c r="B17" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="F17" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="G17" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="H17" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="J17" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="K17" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="L17" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="N17" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="O17" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="P17" s="11" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="18" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="B18" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="C18" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="D18" s="12"/>
+      <c r="F18" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="G18" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="H18" s="12"/>
+      <c r="J18" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="K18" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="L18" s="12"/>
+      <c r="N18" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="O18" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="P18" s="12"/>
+    </row>
+    <row r="19" spans="2:16" ht="15" x14ac:dyDescent="0.2">
+      <c r="B19" s="27" t="s">
+        <v>16</v>
+      </c>
+      <c r="C19" s="27"/>
+      <c r="D19" s="27"/>
+      <c r="F19" s="27" t="s">
+        <v>16</v>
+      </c>
+      <c r="G19" s="27"/>
+      <c r="H19" s="27"/>
+      <c r="J19" s="27" t="s">
+        <v>16</v>
+      </c>
+      <c r="K19" s="27"/>
+      <c r="L19" s="27"/>
+      <c r="N19" s="27" t="s">
+        <v>16</v>
+      </c>
+      <c r="O19" s="27"/>
+      <c r="P19" s="27"/>
+    </row>
+    <row r="20" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="B20" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="C20" s="28"/>
+      <c r="D20" s="28"/>
+      <c r="F20" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="G20" s="28"/>
+      <c r="H20" s="28"/>
+      <c r="J20" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="K20" s="28"/>
+      <c r="L20" s="28"/>
+      <c r="N20" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="O20" s="28"/>
+      <c r="P20" s="28"/>
+    </row>
+    <row r="21" spans="2:16" ht="15" x14ac:dyDescent="0.2">
+      <c r="B21" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="D21" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="F21" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="G21" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="H21" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="J21" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="K21" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="L21" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="N21" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="O21" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="P21" s="11" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="22" spans="2:16" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="B22" s="13">
+        <v>5</v>
+      </c>
+      <c r="C22" s="13">
+        <v>8</v>
+      </c>
+      <c r="D22" s="12"/>
+      <c r="F22" s="13">
+        <v>5</v>
+      </c>
+      <c r="G22" s="13">
+        <v>8</v>
+      </c>
+      <c r="H22" s="12"/>
+      <c r="J22" s="13">
+        <v>5</v>
+      </c>
+      <c r="K22" s="13">
+        <v>8</v>
+      </c>
+      <c r="L22" s="12"/>
+      <c r="N22" s="13">
+        <v>5</v>
+      </c>
+      <c r="O22" s="13">
+        <v>8</v>
+      </c>
+      <c r="P22" s="12"/>
+    </row>
+    <row r="23" spans="2:16" ht="15" x14ac:dyDescent="0.2">
+      <c r="B23" s="27" t="s">
+        <v>155</v>
+      </c>
+      <c r="C23" s="27"/>
+      <c r="D23" s="27"/>
+      <c r="F23" s="27" t="s">
+        <v>155</v>
+      </c>
+      <c r="G23" s="27"/>
+      <c r="H23" s="27"/>
+      <c r="J23" s="27" t="s">
+        <v>155</v>
+      </c>
+      <c r="K23" s="27"/>
+      <c r="L23" s="27"/>
+      <c r="N23" s="27" t="s">
+        <v>155</v>
+      </c>
+      <c r="O23" s="27"/>
+      <c r="P23" s="27"/>
+    </row>
+    <row r="24" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="B24" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C24" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="D24" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="F24" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="G24" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="H24" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="J24" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="K24" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="L24" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="N24" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="O24" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="P24" s="14" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="25" spans="2:16" ht="51" x14ac:dyDescent="0.2">
+      <c r="B25" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="D25" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="F25" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="G25" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="H25" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="J25" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="K25" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="L25" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="N25" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="O25" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="P25" s="12" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="26" spans="2:16" ht="51" x14ac:dyDescent="0.2">
+      <c r="B26" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="D26" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="F26" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="G26" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="H26" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="J26" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="K26" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="L26" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="N26" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="O26" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="P26" s="12" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="27" spans="2:16" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="B27" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="D27" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="F27" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="G27" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="H27" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="J27" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="K27" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="L27" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="N27" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="O27" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="P27" s="12" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="28" spans="2:16" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="B28" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="C28" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>181</v>
+      </c>
+      <c r="F28" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="G28" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="H28" s="12" t="s">
+        <v>181</v>
+      </c>
+      <c r="J28" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="K28" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="L28" s="12" t="s">
+        <v>181</v>
+      </c>
+      <c r="N28" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="O28" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="P28" s="12" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="29" spans="2:16" ht="15" x14ac:dyDescent="0.2">
+      <c r="B29" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="C29" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="D29" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="F29" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="G29" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="H29" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="J29" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="K29" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="L29" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="N29" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="O29" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="P29" s="11" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="30" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="B30" s="12"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="12"/>
+      <c r="F30" s="12"/>
+      <c r="G30" s="12"/>
+      <c r="H30" s="12"/>
+      <c r="J30" s="12"/>
+      <c r="K30" s="12"/>
+      <c r="L30" s="12"/>
+      <c r="N30" s="12"/>
+      <c r="O30" s="12"/>
+      <c r="P30" s="12"/>
+    </row>
+  </sheetData>
+  <mergeCells count="27">
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="F20:H20"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="F23:H23"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="N19:P19"/>
+    <mergeCell ref="J20:L20"/>
+    <mergeCell ref="N20:P20"/>
+    <mergeCell ref="J23:L23"/>
+    <mergeCell ref="N23:P23"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="F8:H8"/>
+    <mergeCell ref="J8:L8"/>
+    <mergeCell ref="N8:P8"/>
+    <mergeCell ref="R8:T8"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="F19:H19"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="N4:P4"/>
+    <mergeCell ref="R4:T4"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="F5:H5"/>
+    <mergeCell ref="J5:L5"/>
+    <mergeCell ref="N5:P5"/>
+    <mergeCell ref="R5:T5"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E290632-FEC5-4D17-94B6-28724497CC62}">
+  <dimension ref="B1:H16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="17.7109375" customWidth="1"/>
+    <col min="3" max="3" width="30.7109375" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" customWidth="1"/>
+    <col min="6" max="6" width="17.7109375" customWidth="1"/>
+    <col min="7" max="7" width="30.7109375" customWidth="1"/>
+    <col min="8" max="8" width="17.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="2:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="B2" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="H2" s="11" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="B3" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="D3" s="12"/>
+      <c r="F3" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="G3" s="15" t="s">
+        <v>139</v>
+      </c>
+      <c r="H3" s="12"/>
+    </row>
+    <row r="4" spans="2:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="B4" s="27" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="27"/>
+      <c r="D4" s="27"/>
+      <c r="F4" s="27" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="27"/>
+      <c r="H4" s="27"/>
+    </row>
+    <row r="5" spans="2:8" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B5" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="F5" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="G5" s="28"/>
+      <c r="H5" s="28"/>
+    </row>
+    <row r="6" spans="2:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="B6" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="H6" s="11" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="B7" s="13">
+        <v>5</v>
+      </c>
+      <c r="C7" s="13">
+        <v>8</v>
+      </c>
+      <c r="D7" s="12"/>
+      <c r="F7" s="13">
+        <v>5</v>
+      </c>
+      <c r="G7" s="13">
+        <v>8</v>
+      </c>
+      <c r="H7" s="12"/>
+    </row>
+    <row r="8" spans="2:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="B8" s="27" t="s">
+        <v>155</v>
+      </c>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+      <c r="F8" s="27" t="s">
+        <v>155</v>
+      </c>
+      <c r="G8" s="27"/>
+      <c r="H8" s="27"/>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B9" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="F9" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="G9" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="H9" s="14" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="B10" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="H10" s="12" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="11" spans="2:8" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="B11" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="G11" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="H11" s="12" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="12" spans="2:8" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="B12" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="G12" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="H12" s="12" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="B13" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>181</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="G13" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="H13" s="12" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="B14" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="G14" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="H14" s="11" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B15" s="12"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
+    </row>
+    <row r="16" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B16" s="16"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="16"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="16"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="F8:H8"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="F5:H5"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>